<commit_message>
:bug: fix: update BASE_COMMISS_FINAL.xlsx with changes in wrong Cod_Cargo: GERENTE QUIOSQUE from 150 to 250
</commit_message>
<xml_diff>
--- a/docs/dom-rock/BASE_COMMISS_FINAL.xlsx
+++ b/docs/dom-rock/BASE_COMMISS_FINAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\FATEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JONIELRODRIGUESDEOLI\Documents\GitHub2\phoenix\API_6_backend\docs\dom-rock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A6965D-E7A0-4614-9C49-69A4C43DB116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30973BC1-F5F7-46AE-9817-B4CDAD7723CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E0DD8414-08D5-4359-B51A-7CBB5556B1F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0DD8414-08D5-4359-B51A-7CBB5556B1F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Commission" sheetId="1" r:id="rId1"/>
@@ -957,16 +957,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F791FF-9814-4BAE-A5D7-54992A4C40F4}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.109375" customWidth="1"/>
-    <col min="2" max="2" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" customWidth="1"/>
-    <col min="4" max="4" width="33.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -983,7 +983,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>10</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>10</v>
       </c>
@@ -1034,7 +1034,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>10</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>10</v>
       </c>
@@ -1059,7 +1059,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>1</v>
@@ -1068,7 +1068,7 @@
         <v>7.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>20</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>20</v>
       </c>
@@ -1102,7 +1102,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>20</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>20</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>1</v>
@@ -1153,7 +1153,7 @@
         <v>1.2500000000000001E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>30</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>30</v>
       </c>
@@ -1187,7 +1187,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>30</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>30</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>30</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>7</v>
       </c>
       <c r="C16" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>1</v>
@@ -1238,7 +1238,7 @@
         <v>2.5000000000000001E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>40</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>40</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>40</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>40</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>40</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>3</v>
       </c>
       <c r="C21" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>1</v>
@@ -1323,7 +1323,7 @@
         <v>1.7500000000000002E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>50</v>
       </c>
@@ -1340,7 +1340,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>50</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>50</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>50</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>50</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>6</v>
       </c>
       <c r="C26" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>1</v>
@@ -1408,7 +1408,7 @@
         <v>7.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>60</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>60</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>60</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>60</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>60</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="2">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>1</v>

</xml_diff>